<commit_message>
feat: video processing pipeline with platform fixes and timeout control
- Replace absolute tool paths with PATH-aware commands (yt-dlp, ffmpeg, ffprobe)
- Fix B站 412 error: Chrome UA + Referer header + valid cookies
- Fix YouTube download: fresh cookies + --js-runtimes node + --remote-components ejs:github
- Add extra_args support in PLATFORM_CONFIG for per-platform custom args
- Add --download-timeout / --transcode-timeout / --transcribe-timeout (default 600/300/600s)
- Timeout triggers exponential backoff retry, does NOT block other concurrent tasks
- get_duration() uses ffprobe directly instead of parsing ffmpeg stderr regex
- Full README rewrite: install guide, cookie export steps, platform matrix, troubleshooting
- Update Excel split sheets
</commit_message>
<xml_diff>
--- a/export_2026-06-10_split-base.xlsx
+++ b/export_2026-06-10_split-base.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12525" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="12525" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="PDF资源" sheetId="1" r:id="rId1"/>
@@ -4996,11 +4996,13 @@
   <dimension ref="A1:Q73"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="5" max="5" width="24.625" customWidth="1"/>
-    <col min="6" max="6" width="28.25" customWidth="1"/>
+    <col min="5" max="5" width="48.375" customWidth="1"/>
+    <col min="6" max="6" width="23.875" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="11" max="11" width="14.25" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="8" max="8" width="9.375" customWidth="1"/>
+    <col min="11" max="11" width="18.25" customWidth="1"/>
+    <col min="12" max="12" width="20.375" customWidth="1"/>
+    <col min="13" max="14" width="17.125" customWidth="1"/>
     <col min="15" max="15" width="15.625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>